<commit_message>
Replaced the previously used Excel workbook file SHA256 hash value with Excel workbook file metadata Length and LastWriteTimestamp for file change detection.
</commit_message>
<xml_diff>
--- a/SampleExcelFiles/LongFilenameDataImportTestMetadata.xlsx
+++ b/SampleExcelFiles/LongFilenameDataImportTestMetadata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/External/Projects/GitHub/UniSharper.Data.Metadata/master/SampleExcelFiles/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54E73CA4-034F-CA43-ADC3-ACA6785EB22B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B0C5F8-8D95-6C4C-8C78-AC3C8562EF85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -47,10 +47,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>(1.0, 1.0)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Vector2Int</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -59,10 +55,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>(1, 1)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Vector3</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -392,6 +384,14 @@
   </si>
   <si>
     <t>Key1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(2, 1)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(2.0, 1.0)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -850,283 +850,283 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="O1" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="T1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="U1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="U1" s="1" t="s">
-        <v>72</v>
-      </c>
       <c r="V1" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="30" customHeight="1">
       <c r="A2" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>23</v>
-      </c>
       <c r="K2" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="T2" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="U2" s="3" t="s">
-        <v>71</v>
-      </c>
       <c r="V2" s="3" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="30" customHeight="1">
       <c r="A3" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="J3" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="4" t="s">
-        <v>24</v>
-      </c>
       <c r="K3" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="L3" s="4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q3" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="R3" s="4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="U3" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="V3" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="W3" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="30" customHeight="1">
       <c r="A4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>3</v>
-      </c>
       <c r="C4" s="4" t="s">
-        <v>6</v>
+        <v>88</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="S4" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="T4" s="4" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="U4" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="V4" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="W4" s="4" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>